<commit_message>
Funcionalidades mayores en indicadores y resultados. Se separan modularmente los gráficos, se configuran las columnas de cada evaluación o indicador para hacer BI o dashboards
</commit_message>
<xml_diff>
--- a/data/database/indicator_metrics.xlsx
+++ b/data/database/indicator_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,22 @@
         <v>5</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance Results Page with Dynamic Role Labels and Achievement Levels
- Updated KPI cards to display dynamic labels based on roleLabels.
- Passed roleLabels and achievement_levels to various components including GraficoDistribucionNiveles, GraficoHabilidades, and TablaAlumnos for improved data representation.
- Modified MetricToggle to utilize dynamic labels for metrics.
- Enhanced data processing to include roleLabels and achievement_levels from the result object.
- Adjusted chart components to handle dynamic achievement levels and improve visual representation of student performance.
- Refactored TablaResumenCursos to dynamically generate headers based on available achievement levels.
</commit_message>
<xml_diff>
--- a/data/database/indicator_metrics.xlsx
+++ b/data/database/indicator_metrics.xlsx
@@ -442,34 +442,34 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixex data visualizations for course level distribution, including bar and pie charts, a summary table, and supporting data files.
</commit_message>
<xml_diff>
--- a/data/database/indicator_metrics.xlsx
+++ b/data/database/indicator_metrics.xlsx
@@ -442,34 +442,34 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor dashboardRenderer and plotly charts for improved layout handling and error reporting
- Updated dashboardRenderer to show an empty placeholder for indicators without a configured layout instead of using a fallback layout.
- Introduced a MissingConfigError component to display missing fields for Plotly components, enhancing error visibility.
- Added support for dynamic valueField toggling in ItemRenderer for components with multiple values.
- Refactored PlotlyWrapper and various chart components (BarByGroup, HorizontalBarByDimension, etc.) to utilize formatStr for dynamic y-axis and x-axis properties.
- Improved handling of percentage formatting across multiple chart types.
- Cleaned up legacy code and comments for better readability and maintainability.
</commit_message>
<xml_diff>
--- a/data/database/indicator_metrics.xlsx
+++ b/data/database/indicator_metrics.xlsx
@@ -442,42 +442,42 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>